<commit_message>
Exclude COŞ_D, EFG and Lüx maşa rows per manufacturer request
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AgVSEcAK2zrsMFYcFqH75Y
</commit_message>
<xml_diff>
--- a/uretici/Tum_Urunler_Barkod_Listesi.xlsx
+++ b/uretici/Tum_Urunler_Barkod_Listesi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Özet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tüm Ürünler'!$A$1:$I$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tüm Ürünler'!$A$1:$I$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I216"/>
+  <dimension ref="A1:I213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1410,11 +1410,7 @@
           <t>DNC-023</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D023</t>
-        </is>
-      </c>
+      <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>1 AD TİTANİUM İSTİRİDYE ŞEKER MAŞASI</t>
@@ -1882,11 +1878,7 @@
           <t>DNC-036</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D036</t>
-        </is>
-      </c>
+      <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Damla Makarna Maşası</t>
@@ -1925,11 +1917,7 @@
           <t>DNC-037</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D037</t>
-        </is>
-      </c>
+      <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Damla Salata Maşası</t>
@@ -1968,11 +1956,7 @@
           <t>DNC-038</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D038</t>
-        </is>
-      </c>
+      <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Damla Pasta Maşası</t>
@@ -2319,11 +2303,7 @@
           <t>DNC-048</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D048</t>
-        </is>
-      </c>
+      <c r="B47" s="2" t="inlineStr"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
           <t>6'LI İSTİRİDYE ÇAY  KAŞIK SADE</t>
@@ -5045,11 +5025,7 @@
           <t>DNC-120</t>
         </is>
       </c>
-      <c r="B117" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D120</t>
-        </is>
-      </c>
+      <c r="B117" s="2" t="inlineStr"/>
       <c r="C117" s="2" t="inlineStr">
         <is>
           <t>Kelebek Maşa Seti</t>
@@ -5166,11 +5142,7 @@
           <t>DNC-123</t>
         </is>
       </c>
-      <c r="B120" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D123</t>
-        </is>
-      </c>
+      <c r="B120" s="2" t="inlineStr"/>
       <c r="C120" s="2" t="inlineStr">
         <is>
           <t>Kelebek Maşa Seti</t>
@@ -5287,14 +5259,10 @@
           <t>DNC-126</t>
         </is>
       </c>
-      <c r="B123" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D126</t>
-        </is>
-      </c>
+      <c r="B123" s="2" t="inlineStr"/>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>COŞ_D 126 GOLD BEYAZ KELEBEKLİ  MAŞA SET</t>
+          <t>DNC_126 GOLD BEYAZ KELEBEKLİ  MAŞA SET</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr"/>
@@ -5400,11 +5368,7 @@
           <t>DNC-129</t>
         </is>
       </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>EFG_129</t>
-        </is>
-      </c>
+      <c r="B126" s="2" t="inlineStr"/>
       <c r="C126" s="2" t="inlineStr">
         <is>
           <t>2,Lİ PASTA SET GOLD TÜY</t>
@@ -5443,11 +5407,7 @@
           <t>DNC-130</t>
         </is>
       </c>
-      <c r="B127" s="2" t="inlineStr">
-        <is>
-          <t>EFG_130</t>
-        </is>
-      </c>
+      <c r="B127" s="2" t="inlineStr"/>
       <c r="C127" s="2" t="inlineStr">
         <is>
           <t>2,Lİ PASTA SET GÜMÜŞ TÜY</t>
@@ -5564,11 +5524,7 @@
           <t>DNC-133</t>
         </is>
       </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D133</t>
-        </is>
-      </c>
+      <c r="B130" s="2" t="inlineStr"/>
       <c r="C130" s="2" t="inlineStr">
         <is>
           <t>3'LÜ  GÜMÜŞ MAŞA BEYAZ  KELEBEK DEKORLU</t>
@@ -6227,14 +6183,10 @@
           <t>DNC-150</t>
         </is>
       </c>
-      <c r="B147" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D150</t>
-        </is>
-      </c>
+      <c r="B147" s="2" t="inlineStr"/>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>COŞ_D 150  ŞEKER  MAŞASI 1 ADET</t>
+          <t>DNC-150  ŞEKER  MAŞASI 1 ADET</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr"/>
@@ -6617,11 +6569,7 @@
           <t>DNC-160</t>
         </is>
       </c>
-      <c r="B157" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D160</t>
-        </is>
-      </c>
+      <c r="B157" s="2" t="inlineStr"/>
       <c r="C157" s="2" t="inlineStr">
         <is>
           <t>Okyanus Sos Kepçesi</t>
@@ -6699,11 +6647,7 @@
           <t>DNC-162</t>
         </is>
       </c>
-      <c r="B159" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D162</t>
-        </is>
-      </c>
+      <c r="B159" s="2" t="inlineStr"/>
       <c r="C159" s="2" t="inlineStr">
         <is>
           <t>Okyanus Sos Servis Kaşığı</t>
@@ -6742,11 +6686,7 @@
           <t>DNC-163</t>
         </is>
       </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D163</t>
-        </is>
-      </c>
+      <c r="B160" s="2" t="inlineStr"/>
       <c r="C160" s="2" t="inlineStr">
         <is>
           <t>Okyanus Sos Spatulası</t>
@@ -6824,11 +6764,7 @@
           <t>DNC-165</t>
         </is>
       </c>
-      <c r="B162" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D165</t>
-        </is>
-      </c>
+      <c r="B162" s="2" t="inlineStr"/>
       <c r="C162" s="2" t="inlineStr">
         <is>
           <t>Okyanus 5'li Sos Servis Seti</t>
@@ -6867,11 +6803,7 @@
           <t>DNC-166</t>
         </is>
       </c>
-      <c r="B163" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D166</t>
-        </is>
-      </c>
+      <c r="B163" s="2" t="inlineStr"/>
       <c r="C163" s="2" t="inlineStr">
         <is>
           <t>Okyanus Sos Kepçesi</t>
@@ -6900,7 +6832,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>8683613550661 başka üründe de var: kodsuz satır; Sitedeki barkod teyit edilene kadar şüpheli</t>
+          <t>8683613550661 başka üründe de var: kodsuz: ŞAHANE HOME 36 PRÇ TİTANİUM Ç.K.B SET; Sitedeki barkod teyit edilene kadar şüpheli</t>
         </is>
       </c>
     </row>
@@ -6949,11 +6881,7 @@
           <t>DNC-168</t>
         </is>
       </c>
-      <c r="B165" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D168</t>
-        </is>
-      </c>
+      <c r="B165" s="2" t="inlineStr"/>
       <c r="C165" s="2" t="inlineStr">
         <is>
           <t>Okyanus Sos Servis Kaşığı</t>
@@ -6992,11 +6920,7 @@
           <t>DNC-169</t>
         </is>
       </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D169</t>
-        </is>
-      </c>
+      <c r="B166" s="2" t="inlineStr"/>
       <c r="C166" s="2" t="inlineStr">
         <is>
           <t>Okyanus Sos Spatulası</t>
@@ -7074,11 +6998,7 @@
           <t>DNC-171</t>
         </is>
       </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D171</t>
-        </is>
-      </c>
+      <c r="B168" s="2" t="inlineStr"/>
       <c r="C168" s="2" t="inlineStr">
         <is>
           <t>Okyanus 5'li Sos Servis Seti</t>
@@ -7425,11 +7345,7 @@
           <t>DNC-180</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D180</t>
-        </is>
-      </c>
+      <c r="B177" s="2" t="inlineStr"/>
       <c r="C177" s="2" t="inlineStr">
         <is>
           <t>İSTİRİDYE GOLD ÇAY KAŞIK 6,LI</t>
@@ -7468,11 +7384,7 @@
           <t>DNC-181</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D181</t>
-        </is>
-      </c>
+      <c r="B178" s="2" t="inlineStr"/>
       <c r="C178" s="2" t="inlineStr">
         <is>
           <t>DNC_181 ORKİDE ÇAY KAŞIK 6,LI SADE</t>
@@ -7932,11 +7844,7 @@
           <t>DNC-193</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D193</t>
-        </is>
-      </c>
+      <c r="B190" s="2" t="inlineStr"/>
       <c r="C190" s="2" t="inlineStr">
         <is>
           <t>SALATA MAŞASI TİTANİUM</t>
@@ -7975,11 +7883,7 @@
           <t>DNC-194</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D194</t>
-        </is>
-      </c>
+      <c r="B191" s="2" t="inlineStr"/>
       <c r="C191" s="2" t="inlineStr">
         <is>
           <t>PASTA MAŞASI TİTANİUM</t>
@@ -8018,11 +7922,7 @@
           <t>DNC-195</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
-        <is>
-          <t>COŞ_D195</t>
-        </is>
-      </c>
+      <c r="B192" s="2" t="inlineStr"/>
       <c r="C192" s="2" t="inlineStr">
         <is>
           <t>MAKARNA MAŞASI TİTANİUM</t>
@@ -8100,11 +8000,7 @@
           <t>DNC-197</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
-        <is>
-          <t>EFG_197</t>
-        </is>
-      </c>
+      <c r="B194" s="2" t="inlineStr"/>
       <c r="C194" s="2" t="inlineStr">
         <is>
           <t>5,Lİ GÜMÜŞ TÜY SOS SERVİS SET</t>
@@ -8182,11 +8078,7 @@
           <t>DNC-199</t>
         </is>
       </c>
-      <c r="B196" s="2" t="inlineStr">
-        <is>
-          <t>EFG_199</t>
-        </is>
-      </c>
+      <c r="B196" s="2" t="inlineStr"/>
       <c r="C196" s="2" t="inlineStr">
         <is>
           <t>5,Lİ GOLD TÜY SOS SERVİS SET</t>
@@ -8420,11 +8312,7 @@
           <t>DNC-205</t>
         </is>
       </c>
-      <c r="B202" s="2" t="inlineStr">
-        <is>
-          <t>EFG_205</t>
-        </is>
-      </c>
+      <c r="B202" s="2" t="inlineStr"/>
       <c r="C202" s="2" t="inlineStr">
         <is>
           <t>Zerafet 5'li Sunum Servis Seti</t>
@@ -8463,11 +8351,7 @@
           <t>DNC-206</t>
         </is>
       </c>
-      <c r="B203" s="2" t="inlineStr">
-        <is>
-          <t>EFG_206</t>
-        </is>
-      </c>
+      <c r="B203" s="2" t="inlineStr"/>
       <c r="C203" s="2" t="inlineStr">
         <is>
           <t>Zerafet 5'li Sunum Servis Seti</t>
@@ -8576,11 +8460,7 @@
           <t>DNC-209</t>
         </is>
       </c>
-      <c r="B206" s="2" t="inlineStr">
-        <is>
-          <t>EFG_209</t>
-        </is>
-      </c>
+      <c r="B206" s="2" t="inlineStr"/>
       <c r="C206" s="2" t="inlineStr">
         <is>
           <t>Zerafet 5'li Sunum Servis Seti</t>
@@ -8732,20 +8612,20 @@
           <t>(kodsuz)</t>
         </is>
       </c>
-      <c r="B210" s="2" t="inlineStr">
-        <is>
-          <t>805</t>
-        </is>
-      </c>
+      <c r="B210" s="2" t="inlineStr"/>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>LÜX MAKARNA MAŞASI KOD 805</t>
-        </is>
-      </c>
-      <c r="D210" s="3" t="inlineStr"/>
+          <t>Gümüş 84 Parça Çatal-Kaşık-Bıçak Seti</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>8683581657751</t>
+        </is>
+      </c>
       <c r="E210" s="3" t="inlineStr">
         <is>
-          <t>8681198062265</t>
+          <t>8683581657751</t>
         </is>
       </c>
       <c r="F210" s="2" t="inlineStr">
@@ -8761,7 +8641,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>8681198062265 Dincel önekiyle başlamıyor (başka firmanın ürünü olabilir); DNC ürün kodu yok; Yalnızca yeni listede</t>
+          <t>DNC ürün kodu yok</t>
         </is>
       </c>
     </row>
@@ -8771,20 +8651,20 @@
           <t>(kodsuz)</t>
         </is>
       </c>
-      <c r="B211" s="2" t="inlineStr">
-        <is>
-          <t>806</t>
-        </is>
-      </c>
+      <c r="B211" s="2" t="inlineStr"/>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>LÜX PASTA MAŞASI KOD 806</t>
-        </is>
-      </c>
-      <c r="D211" s="3" t="inlineStr"/>
+          <t>Gümüş 89 Parça Çatal-Kaşık-Bıçak Seti</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>8683581657768</t>
+        </is>
+      </c>
       <c r="E211" s="3" t="inlineStr">
         <is>
-          <t>8681198062272</t>
+          <t>8683581657768</t>
         </is>
       </c>
       <c r="F211" s="2" t="inlineStr">
@@ -8800,7 +8680,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>8681198062272 Dincel önekiyle başlamıyor (başka firmanın ürünü olabilir); DNC ürün kodu yok; Yalnızca yeni listede</t>
+          <t>DNC ürün kodu yok</t>
         </is>
       </c>
     </row>
@@ -8810,20 +8690,16 @@
           <t>(kodsuz)</t>
         </is>
       </c>
-      <c r="B212" s="2" t="inlineStr">
-        <is>
-          <t>807</t>
-        </is>
-      </c>
+      <c r="B212" s="2" t="inlineStr"/>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>LÜX SALATA MAŞASI KOD 807</t>
+          <t>ŞAHANE HOME 36 PRÇ TİTANİUM Ç.K.B SET</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr"/>
       <c r="E212" s="3" t="inlineStr">
         <is>
-          <t>8681198062289</t>
+          <t>8683613550661</t>
         </is>
       </c>
       <c r="F212" s="2" t="inlineStr">
@@ -8839,7 +8715,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>8681198062289 Dincel önekiyle başlamıyor (başka firmanın ürünü olabilir); DNC ürün kodu yok; Yalnızca yeni listede</t>
+          <t>8683613550661 başka üründe de var: DNC-166; DNC ürün kodu yok; Yalnızca yeni listede</t>
         </is>
       </c>
     </row>
@@ -8852,17 +8728,13 @@
       <c r="B213" s="2" t="inlineStr"/>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>Gümüş 84 Parça Çatal-Kaşık-Bıçak Seti</t>
-        </is>
-      </c>
-      <c r="D213" s="3" t="inlineStr">
-        <is>
-          <t>8683581657751</t>
-        </is>
-      </c>
+          <t>SARAY SOS KEPÇE</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="inlineStr"/>
       <c r="E213" s="3" t="inlineStr">
         <is>
-          <t>8683581657751</t>
+          <t>8699182306042</t>
         </is>
       </c>
       <c r="F213" s="2" t="inlineStr">
@@ -8878,121 +8750,12 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>DNC ürün kodu yok</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="2" t="inlineStr">
-        <is>
-          <t>(kodsuz)</t>
-        </is>
-      </c>
-      <c r="B214" s="2" t="inlineStr"/>
-      <c r="C214" s="2" t="inlineStr">
-        <is>
-          <t>Gümüş 89 Parça Çatal-Kaşık-Bıçak Seti</t>
-        </is>
-      </c>
-      <c r="D214" s="3" t="inlineStr">
-        <is>
-          <t>8683581657768</t>
-        </is>
-      </c>
-      <c r="E214" s="3" t="inlineStr">
-        <is>
-          <t>8683581657768</t>
-        </is>
-      </c>
-      <c r="F214" s="2" t="inlineStr">
-        <is>
-          <t>Sitede yok</t>
-        </is>
-      </c>
-      <c r="G214" s="3" t="inlineStr"/>
-      <c r="H214" s="4" t="inlineStr">
-        <is>
-          <t>ÜRETİCİ TEYİDİ GEREKLİ</t>
-        </is>
-      </c>
-      <c r="I214" s="2" t="inlineStr">
-        <is>
-          <t>DNC ürün kodu yok</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" s="2" t="inlineStr">
-        <is>
-          <t>(kodsuz)</t>
-        </is>
-      </c>
-      <c r="B215" s="2" t="inlineStr"/>
-      <c r="C215" s="2" t="inlineStr">
-        <is>
-          <t>ŞAHANE HOME 36 PRÇ TİTANİUM Ç.K.B SET</t>
-        </is>
-      </c>
-      <c r="D215" s="3" t="inlineStr"/>
-      <c r="E215" s="3" t="inlineStr">
-        <is>
-          <t>8683613550661</t>
-        </is>
-      </c>
-      <c r="F215" s="2" t="inlineStr">
-        <is>
-          <t>Sitede yok</t>
-        </is>
-      </c>
-      <c r="G215" s="3" t="inlineStr"/>
-      <c r="H215" s="4" t="inlineStr">
-        <is>
-          <t>ÜRETİCİ TEYİDİ GEREKLİ</t>
-        </is>
-      </c>
-      <c r="I215" s="2" t="inlineStr">
-        <is>
-          <t>8683613550661 başka üründe de var: DNC-166; DNC ürün kodu yok; Yalnızca yeni listede</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" s="2" t="inlineStr">
-        <is>
-          <t>(kodsuz)</t>
-        </is>
-      </c>
-      <c r="B216" s="2" t="inlineStr"/>
-      <c r="C216" s="2" t="inlineStr">
-        <is>
-          <t>SARAY SOS KEPÇE</t>
-        </is>
-      </c>
-      <c r="D216" s="3" t="inlineStr"/>
-      <c r="E216" s="3" t="inlineStr">
-        <is>
-          <t>8699182306042</t>
-        </is>
-      </c>
-      <c r="F216" s="2" t="inlineStr">
-        <is>
-          <t>Sitede yok</t>
-        </is>
-      </c>
-      <c r="G216" s="3" t="inlineStr"/>
-      <c r="H216" s="4" t="inlineStr">
-        <is>
-          <t>ÜRETİCİ TEYİDİ GEREKLİ</t>
-        </is>
-      </c>
-      <c r="I216" s="2" t="inlineStr">
-        <is>
           <t>8699182306042 Dincel önekiyle başlamıyor (başka firmanın ürünü olabilir); DNC ürün kodu yok; Yalnızca yeni listede</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I216"/>
+  <autoFilter ref="A1:I213"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9029,7 +8792,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>COUNTIF('Tüm Ürünler'!$H$2:$H$216,"TAMAM")</f>
+        <f>COUNTIF('Tüm Ürünler'!$H$2:$H$213,"TAMAM")</f>
         <v/>
       </c>
     </row>
@@ -9040,7 +8803,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF('Tüm Ürünler'!$H$2:$H$216,"ÜRETİCİ TEYİDİ GEREKLİ")</f>
+        <f>COUNTIF('Tüm Ürünler'!$H$2:$H$213,"ÜRETİCİ TEYİDİ GEREKLİ")</f>
         <v/>
       </c>
     </row>
@@ -9051,7 +8814,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF('Tüm Ürünler'!$H$2:$H$216,"BARKOD YOK")</f>
+        <f>COUNTIF('Tüm Ürünler'!$H$2:$H$213,"BARKOD YOK")</f>
         <v/>
       </c>
     </row>
@@ -9062,7 +8825,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTA('Tüm Ürünler'!$A$2:$A$216)</f>
+        <f>COUNTA('Tüm Ürünler'!$A$2:$A$213)</f>
         <v/>
       </c>
     </row>
@@ -9076,7 +8839,7 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>COUNTIF('Tüm Ürünler'!$F$2:$F$216,"Barkod yazılı*")</f>
+        <f>COUNTIF('Tüm Ürünler'!$F$2:$F$213,"Barkod yazılı*")</f>
         <v/>
       </c>
     </row>
@@ -9087,7 +8850,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF('Tüm Ürünler'!$F$2:$F$216,"Sitede var, barkod boş")</f>
+        <f>COUNTIF('Tüm Ürünler'!$F$2:$F$213,"Sitede var, barkod boş")</f>
         <v/>
       </c>
     </row>
@@ -9098,7 +8861,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF('Tüm Ürünler'!$F$2:$F$216,"Sitede yok")</f>
+        <f>COUNTIF('Tüm Ürünler'!$F$2:$F$213,"Sitede yok")</f>
         <v/>
       </c>
     </row>
@@ -9109,14 +8872,14 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIFS('Tüm Ürünler'!$F$2:$F$216,"Barkod yazılı*",'Tüm Ürünler'!$H$2:$H$216,"ÜRETİCİ TEYİDİ GEREKLİ")</f>
+        <f>COUNTIFS('Tüm Ürünler'!$F$2:$F$213,"Barkod yazılı*",'Tüm Ürünler'!$H$2:$H$213,"ÜRETİCİ TEYİDİ GEREKLİ")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Kaynaklar: İlk liste = Dincel_Celik_Urun_Listesi_Tum_DNC_Doldurulmus.xlsx; Yeni liste = barkod_listesi.xlsx; Site = dincelcelik.com.tr, 04.10.2026 itibarıyla. COŞ_D / EFG kodları aynı numaralı DNC koduyla aynı ürün kabul edildi.</t>
+          <t>Kaynaklar: İlk liste = Dincel_Celik_Urun_Listesi_Tum_DNC_Doldurulmus.xlsx; Yeni liste = barkod_listesi.xlsx; Site = dincelcelik.com.tr, 04.10.2026 itibarıyla. Yeni listedeki COŞ_D, EFG ve Lüx maşa 805/806/807 satırları üreticinin isteğiyle çıkarıldı.</t>
         </is>
       </c>
     </row>

</xml_diff>